<commit_message>
Scenario 1 GT evidence files updated
</commit_message>
<xml_diff>
--- a/Applied-Research Project/05-Implementation/02_Atomic_Red_Teams_Attack_Scenarios/01_T1059.003_Windows_Command_Shell/02_Ground_Truth/Scenario_1.xlsx
+++ b/Applied-Research Project/05-Implementation/02_Atomic_Red_Teams_Attack_Scenarios/01_T1059.003_Windows_Command_Shell/02_Ground_Truth/Scenario_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\darra\Documents\GitHub\applied-research-project\Applied-Research Project\05-Implementation\02_Atomic_Red_Teams_Attack_Scenarios\01_T1059.003_Windows_Command_Shell\02_Ground_Truth\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37A0B830-1E97-4532-B3F0-F710E381C714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D83434D2-06A8-4A8F-88C1-8E726D6FA1A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{6EDD1CA0-2A49-4EF7-89EA-F85052302D67}"/>
   </bookViews>
@@ -71,9 +71,6 @@
     <t>Evidence files</t>
   </si>
   <si>
-    <t>Test_1_Archives.json / Test_1_Alerts.json</t>
-  </si>
-  <si>
     <t>GT ID</t>
   </si>
   <si>
@@ -239,6 +236,9 @@
 • EventRecordID 15251 records cmd.exe PID 8188 using /c against T1059.003_script.bat
 • EventRecordID 15251 identifies PowerShell PID 1212 as the direct parent
 • No supplied telemetry contains Set-Content, the batch-file contents or stdout</t>
+  </si>
+  <si>
+    <t>Scenario_1_Archives.json / Scenario_1_Alerts.json</t>
   </si>
 </sst>
 </file>
@@ -728,7 +728,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C4" s="8"/>
       <c r="D4" s="7"/>
@@ -739,7 +739,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C5" s="8"/>
       <c r="D5" s="7"/>
@@ -750,7 +750,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C6" s="8"/>
       <c r="D6" s="7"/>
@@ -761,7 +761,7 @@
         <v>9</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>10</v>
+        <v>47</v>
       </c>
       <c r="C7" s="8"/>
       <c r="D7" s="7"/>
@@ -769,121 +769,121 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="C8" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="D8" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="E8" s="10" t="s">
         <v>14</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="5" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="C9" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" s="12" t="s">
         <v>17</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="E9" s="12" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="5" customFormat="1" ht="145.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="5" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="12" t="s">
         <v>20</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="D11" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="5" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="5" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C13" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="D13" s="13" t="s">
-        <v>38</v>
-      </c>
       <c r="E13" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="5" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Literature Review update along with rephrasing of Ground Truth
</commit_message>
<xml_diff>
--- a/Applied-Research Project/05-Implementation/02_Atomic_Red_Teams_Attack_Scenarios/01_T1059.003_Windows_Command_Shell/02_Ground_Truth/Scenario_1.xlsx
+++ b/Applied-Research Project/05-Implementation/02_Atomic_Red_Teams_Attack_Scenarios/01_T1059.003_Windows_Command_Shell/02_Ground_Truth/Scenario_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\darra\Documents\GitHub\applied-research-project\Applied-Research Project\05-Implementation\02_Atomic_Red_Teams_Attack_Scenarios\01_T1059.003_Windows_Command_Shell\02_Ground_Truth\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D83434D2-06A8-4A8F-88C1-8E726D6FA1A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5329032-DBEF-40BB-9D6F-08B41522CF30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{6EDD1CA0-2A49-4EF7-89EA-F85052302D67}"/>
   </bookViews>
@@ -227,11 +227,6 @@
 • Execution time: 2026-10-02 14:55:27.411 UTC /  16:55:27.411 (UTC+2)</t>
   </si>
   <si>
-    <t>• Batch-file execution through Windows Command Shell confirmed
-• cmd.exe launched the batch file using /c
-• The commands executed within the batch file and any resulting stdout cannot be determined from the supplied evidence.</t>
-  </si>
-  <si>
     <t>• EventRecordID 15248 records PowerShell PID 1212 using Start-Process against T1059.003_script.bat
 • EventRecordID 15251 records cmd.exe PID 8188 using /c against T1059.003_script.bat
 • EventRecordID 15251 identifies PowerShell PID 1212 as the direct parent
@@ -239,6 +234,11 @@
   </si>
   <si>
     <t>Scenario_1_Archives.json / Scenario_1_Alerts.json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Batch-file execution through Windows Command Shell confirmed
+• cmd.exe launched the batch file using /c
+• Does not make unsupportee claime about successful completion or similar. </t>
   </si>
 </sst>
 </file>
@@ -761,7 +761,7 @@
         <v>9</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C7" s="8"/>
       <c r="D7" s="7"/>
@@ -812,7 +812,7 @@
         <v>35</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E10" s="12" t="s">
         <v>42</v>
@@ -835,7 +835,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:5" s="5" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" s="5" customFormat="1" ht="88.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
         <v>21</v>
       </c>
@@ -843,7 +843,7 @@
         <v>25</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D12" s="13" t="s">
         <v>33</v>
@@ -852,7 +852,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:5" s="5" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" s="5" customFormat="1" ht="101.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
         <v>22</v>
       </c>

</xml_diff>

<commit_message>
Ground Truth Scenario 2 added
</commit_message>
<xml_diff>
--- a/Applied-Research Project/05-Implementation/02_Atomic_Red_Teams_Attack_Scenarios/01_T1059.003_Windows_Command_Shell/02_Ground_Truth/Scenario_1.xlsx
+++ b/Applied-Research Project/05-Implementation/02_Atomic_Red_Teams_Attack_Scenarios/01_T1059.003_Windows_Command_Shell/02_Ground_Truth/Scenario_1.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\darra\Documents\GitHub\applied-research-project\Applied-Research Project\05-Implementation\02_Atomic_Red_Teams_Attack_Scenarios\01_T1059.003_Windows_Command_Shell\02_Ground_Truth\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5329032-DBEF-40BB-9D6F-08B41522CF30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AF78B89-A21C-4AE3-9DFA-813C84C50AE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{6EDD1CA0-2A49-4EF7-89EA-F85052302D67}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6EDD1CA0-2A49-4EF7-89EA-F85052302D67}"/>
   </bookViews>
   <sheets>
-    <sheet name="Test 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Scenario 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -268,19 +268,19 @@
     <font>
       <b/>
       <sz val="11"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -330,6 +330,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="47" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="22" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -341,9 +344,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="22" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -749,7 +749,7 @@
       <c r="A6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="10" t="s">
         <v>31</v>
       </c>
       <c r="C6" s="8"/>
@@ -768,121 +768,121 @@
       <c r="E7" s="7"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="11" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="5" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="12" t="s">
+      <c r="E9" s="13" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="5" customFormat="1" ht="145.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="E10" s="13" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="5" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="13" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="5" customFormat="1" ht="88.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="E12" s="12" t="s">
+      <c r="E12" s="13" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="5" customFormat="1" ht="101.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="D13" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="E13" s="12" t="s">
+      <c r="E13" s="13" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="5" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="E14" s="12" t="s">
+      <c r="E14" s="13" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Scenario 1 re run to remove bat script Mitre Technique name - T1059.003_script.bat changed to Scenario_1_script.bat
</commit_message>
<xml_diff>
--- a/Applied-Research Project/05-Implementation/02_Atomic_Red_Teams_Attack_Scenarios/01_T1059.003_Windows_Command_Shell/02_Ground_Truth/Scenario_1.xlsx
+++ b/Applied-Research Project/05-Implementation/02_Atomic_Red_Teams_Attack_Scenarios/01_T1059.003_Windows_Command_Shell/02_Ground_Truth/Scenario_1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\darra\Documents\GitHub\applied-research-project\Applied-Research Project\05-Implementation\02_Atomic_Red_Teams_Attack_Scenarios\01_T1059.003_Windows_Command_Shell\02_Ground_Truth\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AF78B89-A21C-4AE3-9DFA-813C84C50AE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AE23270-1076-4013-8C2C-9ED9705ECE4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6EDD1CA0-2A49-4EF7-89EA-F85052302D67}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{6EDD1CA0-2A49-4EF7-89EA-F85052302D67}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenario 1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t>Scenario name</t>
   </si>
@@ -92,32 +92,18 @@
     <t>Execution &amp; timing</t>
   </si>
   <si>
-    <t>Sysmon Event ID 1
-EventRecordID 15251
-Wazuh Rule 92004.</t>
-  </si>
-  <si>
     <t>GT2</t>
   </si>
   <si>
     <t>GT3</t>
   </si>
   <si>
-    <t>Sysmon Event ID 1
-EventRecordID 15251
-ProcessGuid {4b2ce92d-c5df-6abf-8104-000000001400}.</t>
-  </si>
-  <si>
     <t>GT4</t>
   </si>
   <si>
     <t>GT5</t>
   </si>
   <si>
-    <t>Sysmon Event ID 1
-EventRecordID 15251.</t>
-  </si>
-  <si>
     <t>GT6</t>
   </si>
   <si>
@@ -139,106 +125,104 @@
     <t>Command and Scripting Interpreter: Windows Command Shell</t>
   </si>
   <si>
-    <t>2026-10-02: 16:50:26.665 - 17:00:27.861</t>
-  </si>
-  <si>
-    <t>• Parent process: PowerShell, PID 1212
-• Child process: cmd.exe, PID 8188
-• User: DESKTOP-5OG7C28\Darragh Casey
-• Integrity level: High
-• TerminalSessionId: 1
-• LogonId: 0xA8D6D</t>
-  </si>
-  <si>
-    <t>• Sysmon Process Create:
-  – cmd.exe
-  – T1059.003_script.bat supplied to /c
-• No supplied telemetry records stdout or the resulting directory-listing text</t>
-  </si>
-  <si>
-    <t>• Sysmon Event ID 1 records:
-  – Parent process
-  – Child process
-  – Process IDs
-  – User account
-  – Integrity level
-  – Session details</t>
-  </si>
-  <si>
-    <t>• PowerShell used Start-Process
-• Target file: T1059.003_script.bat
-• Windows executed the batch file using cmd.exe /c
-• The contents of the batch file cannot be determined from the evidence</t>
-  </si>
-  <si>
-    <t>• Primary execution evidence: Sysmon Event ID 1
-• PowerShell execution: EventRecordID 15248
-• Command-shell execution: EventRecordID 15251
-• Wazuh detection: Rule 92004, level 4
-• Rule 92004 identifies PowerShell spawning Windows Command Shell and maps it to T1059.003</t>
-  </si>
-  <si>
-    <t>• Sysmon Event ID 1: process sequence and process details
-• Wazuh Rule 92004:
-  – Embeds correlated Sysmon process event
-  – Shows Powershell launching cmd.exe</t>
-  </si>
-  <si>
-    <t>• Execution used:
-  – C:\Windows\System32\cmd.exe
-  – /c
-  – T1059.003_script.bat
-• Sequence supported by:
-  – Setup telemetry
-  – Process-creation event
-  – Correlated Wazuh alert</t>
-  </si>
-  <si>
-    <t>• MITRE ATT&amp;CK technique: T1059.003 – Windows Command Shell
-• Tactic: Execution
-• Sequence:
-  – PowerShell launched T1059.003_script.bat using Start-Process.
-  – cmd.exe subsequently executed the batch file using /c.
-  – Wazuh detected the PowerShell-to-command-shell execution and mapped it to T1059.003.
-  - Observable sequence: PowerShell Start-Process → cmd.exe /c on T1059.003_script.bat (15251) → Wazuh Rule 92004 / T1059.003.</t>
-  </si>
-  <si>
-    <t>• Sysmon Process Create:
-  – cmd.exe
-  – PID 8188
-  – Time: 14:55:27.411 UTC
-• Matching Wazuh alert:
-  – 16:55:27.929+0200</t>
-  </si>
-  <si>
-    <t>EventRecordIDs 15248, 15251
-Wazuh Rule 92004.</t>
-  </si>
-  <si>
-    <t>EventRecordID 15248, 15251</t>
-  </si>
-  <si>
-    <t>2026-10-02 14:55:27.411 UTC / 16:55:27.411 (UTC+2)</t>
+    <t>Scenario_1_Archives.json / Scenario_1_Alerts.json</t>
+  </si>
+  <si>
+    <t>2026-10-23: 15:33:26.281–15:41:46.496 (UTC+2)</t>
+  </si>
+  <si>
+    <t>2026-10-23 13:37:27.087 UTC / 15:37:27.087 (UTC+2)</t>
   </si>
   <si>
     <t>• Host: DESKTOP-5OG7C28
 • Technique/test: T1059.003 batch-script execution
-• Executable: cmd.exe
-• Execution time: 2026-10-02 14:55:27.411 UTC /  16:55:27.411 (UTC+2)</t>
-  </si>
-  <si>
-    <t>• EventRecordID 15248 records PowerShell PID 1212 using Start-Process against T1059.003_script.bat
-• EventRecordID 15251 records cmd.exe PID 8188 using /c against T1059.003_script.bat
-• EventRecordID 15251 identifies PowerShell PID 1212 as the direct parent
-• No supplied telemetry contains Set-Content, the batch-file contents or stdout</t>
-  </si>
-  <si>
-    <t>Scenario_1_Archives.json / Scenario_1_Alerts.json</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Batch-file execution through Windows Command Shell confirmed
-• cmd.exe launched the batch file using /c
-• Does not make unsupportee claime about successful completion or similar. </t>
+• Executable: C:\Windows\System32\cmd.exe
+• Execution time: 2026-10-23 13:37:27.087 UTC / 15:37:27.087 (UTC+2)</t>
+  </si>
+  <si>
+    <t>• Sysmon Process Create: cmd.exe, PID 6000, at 13:37:27.087 UTC
+• Matching Wazuh alert at 15:37:27.207+0200
+• PowerShell Start-Process event precedes cmd.exe (13:37:26.282 UTC)</t>
+  </si>
+  <si>
+    <t>• PowerShell used Start-Process
+• Target file: Scenario_1_script.bat (C:\AtomicRedTeam\ExternalPayloads)
+• Windows launched cmd.exe /c with the batch-file path
+• Batch-file contents and stdout are not present in supplied logs</t>
+  </si>
+  <si>
+    <t>• EventRecordID 27944: PowerShell Test-Path check for Scenario_1_script.bat (does not establish its result)
+• EventRecordID 27948: PowerShell PID 4500 invokes Start-Process on the batch file
+• EventRecordID 27950: cmd.exe PID 6000 runs /c with the batch-file path and identifies PID 4500 as its direct parent</t>
+  </si>
+  <si>
+    <t>• Parent process: powershell.exe, PID 4500
+• Child process: cmd.exe, PID 6000
+• User: DESKTOP-5OG7C28\Darragh Casey
+• Integrity level: Medium
+• TerminalSessionId: 1
+• LogonId: 0xFCD57</t>
+  </si>
+  <si>
+    <t>• Sysmon Event ID 1 records PowerShell-to-cmd.exe parent-child linkage
+• ParentProcessGuid: {4b2ce92d-6316-6adb-ae04-000000001a00}
+• Child ProcessGuid: {4b2ce92d-6317-6adb-b004-000000001a00}
+• User, integrity level, session and logon details present</t>
+  </si>
+  <si>
+    <t>• Batch-file invocation through Windows Command Shell confirmed
+• cmd.exe created with /c and Scenario_1_script.bat as the target
+• Successful batch completion, output and side effects cannot be established from supplied telemetry</t>
+  </si>
+  <si>
+    <t>• Sysmon process creation confirms cmd.exe PID 6000 and command line pointing to Scenario_1_script.bat
+• No provided event establishes the script’s contents, stdout, exit code or successful completion</t>
+  </si>
+  <si>
+    <t>• Primary execution evidence: Sysmon Event ID 1
+• PowerShell Start-Process: EventRecordID 27948
+• Command-shell creation: EventRecordID 27950
+• Wazuh detection: Rule 92004, level 4; T1059.003 (Execution)
+• Additional Wazuh alerts: Rule 92213 (level 6) on temporary PowerShell policy-test .ps1 files (27945, 27949); Rule 92217 (level 6) on Defender update executables (27937, 27938). These do not independently confirm malicious execution.</t>
+  </si>
+  <si>
+    <t>• Rule 92004 embeds Sysmon command-shell process creation with PowerShell parent
+• Rule 92213 records PowerShell-created __PSScriptPolicyTest_*.ps1 files in user Temp
+• Rule 92217 records MpCmdRun.exe writing mpam-bce1d755.exe and UpdatePlatform.exe beneath C:\Windows\SystemTemp</t>
+  </si>
+  <si>
+    <t>• PowerShell Test-Path: PID 10880, EventRecordID 27944 (13:37:25.589 UTC)
+• PowerShell Start-Process: PID 4500, EventRecordID 27948 (13:37:26.282 UTC)
+• cmd.exe /c: PID 6000, EventRecordID 27950 (13:37:27.087 UTC)
+• Wazuh Rule 92004: 15:37:27.207+0200</t>
+  </si>
+  <si>
+    <t>Sysmon Event ID 1, EventRecordID 27950 Wazuh Rule 92004
+EventRecordID 27948</t>
+  </si>
+  <si>
+    <t>EventRecordIDs 27944, 27948, 27950</t>
+  </si>
+  <si>
+    <t>Sysmon Event ID 1, EventRecordID 27950
+EventRecordID 27948</t>
+  </si>
+  <si>
+    <t>Sysmon Event ID 1, EventRecordID 27950</t>
+  </si>
+  <si>
+    <t>EventRecordIDs 27950 (Rule 92004), 27945 &amp; 27949 (Rule 92213), 27937 &amp; 27938 (Rule 92217)
+EventRecordID 27948</t>
+  </si>
+  <si>
+    <t>EventRecordIDs 27944, 27948, 27950
+EventRecordID 27950, Wazuh Rule 92004</t>
+  </si>
+  <si>
+    <t>• MITRE ATT&amp;CK technique: T1059.003 – Windows Command Shell
+• Tactic: Execution (from Wazuh Rule 92004)
+• Sequence: PowerShell Test-Path check -- PowerShell Start-Process of Scenario_1_script.bat -- cmd.exe /c Scenario_1_script.bat -- Wazuh Rule 92004 alert
+• The available data does not support successful completion of script actions</t>
   </si>
 </sst>
 </file>
@@ -728,7 +712,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C4" s="8"/>
       <c r="D4" s="7"/>
@@ -739,7 +723,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="C5" s="8"/>
       <c r="D5" s="7"/>
@@ -750,7 +734,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C6" s="8"/>
       <c r="D6" s="7"/>
@@ -761,7 +745,7 @@
         <v>9</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="C7" s="8"/>
       <c r="D7" s="7"/>
@@ -792,98 +776,98 @@
         <v>16</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>17</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="5" customFormat="1" ht="145.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" s="5" customFormat="1" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A11" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" s="14" t="s">
+      <c r="B11" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="14" t="s">
+      <c r="D11" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" s="5" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="E12" s="13" t="s">
         <v>45</v>
-      </c>
-      <c r="E10" s="13" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" s="5" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="D11" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="E11" s="13" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" s="5" customFormat="1" ht="88.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="D12" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E12" s="13" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="5" customFormat="1" ht="101.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" s="5" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" s="5" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A14" s="12" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Prompt tweak and Ground truth refined
</commit_message>
<xml_diff>
--- a/Applied-Research Project/05-Implementation/02_Atomic_Red_Teams_Attack_Scenarios/01_T1059.003_Windows_Command_Shell/02_Ground_Truth/Scenario_1.xlsx
+++ b/Applied-Research Project/05-Implementation/02_Atomic_Red_Teams_Attack_Scenarios/01_T1059.003_Windows_Command_Shell/02_Ground_Truth/Scenario_1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\darra\Documents\GitHub\applied-research-project\Applied-Research Project\05-Implementation\02_Atomic_Red_Teams_Attack_Scenarios\01_T1059.003_Windows_Command_Shell\02_Ground_Truth\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AE23270-1076-4013-8C2C-9ED9705ECE4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8CC07A0-6379-4EB5-BD04-F64141884A94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{6EDD1CA0-2A49-4EF7-89EA-F85052302D67}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6EDD1CA0-2A49-4EF7-89EA-F85052302D67}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenario 1" sheetId="1" r:id="rId1"/>
@@ -179,18 +179,6 @@
 • No provided event establishes the script’s contents, stdout, exit code or successful completion</t>
   </si>
   <si>
-    <t>• Primary execution evidence: Sysmon Event ID 1
-• PowerShell Start-Process: EventRecordID 27948
-• Command-shell creation: EventRecordID 27950
-• Wazuh detection: Rule 92004, level 4; T1059.003 (Execution)
-• Additional Wazuh alerts: Rule 92213 (level 6) on temporary PowerShell policy-test .ps1 files (27945, 27949); Rule 92217 (level 6) on Defender update executables (27937, 27938). These do not independently confirm malicious execution.</t>
-  </si>
-  <si>
-    <t>• Rule 92004 embeds Sysmon command-shell process creation with PowerShell parent
-• Rule 92213 records PowerShell-created __PSScriptPolicyTest_*.ps1 files in user Temp
-• Rule 92217 records MpCmdRun.exe writing mpam-bce1d755.exe and UpdatePlatform.exe beneath C:\Windows\SystemTemp</t>
-  </si>
-  <si>
     <t>• PowerShell Test-Path: PID 10880, EventRecordID 27944 (13:37:25.589 UTC)
 • PowerShell Start-Process: PID 4500, EventRecordID 27948 (13:37:26.282 UTC)
 • cmd.exe /c: PID 6000, EventRecordID 27950 (13:37:27.087 UTC)
@@ -211,10 +199,6 @@
     <t>Sysmon Event ID 1, EventRecordID 27950</t>
   </si>
   <si>
-    <t>EventRecordIDs 27950 (Rule 92004), 27945 &amp; 27949 (Rule 92213), 27937 &amp; 27938 (Rule 92217)
-EventRecordID 27948</t>
-  </si>
-  <si>
     <t>EventRecordIDs 27944, 27948, 27950
 EventRecordID 27950, Wazuh Rule 92004</t>
   </si>
@@ -223,6 +207,21 @@
 • Tactic: Execution (from Wazuh Rule 92004)
 • Sequence: PowerShell Test-Path check -- PowerShell Start-Process of Scenario_1_script.bat -- cmd.exe /c Scenario_1_script.bat -- Wazuh Rule 92004 alert
 • The available data does not support successful completion of script actions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Primary execution evidence: Sysmon Event ID 1
+• PowerShell Start-Process: EventRecordID 27948
+• Command-shell creation: EventRecordID 27950
+• Wazuh detection: Rule 92004, level 4; T1059.003 (Execution)
+</t>
+  </si>
+  <si>
+    <t>EventRecordIDs 27950 (Rule 92004), 27945, 27937 &amp; 27938 (Rule 92217)
+EventRecordID 27948</t>
+  </si>
+  <si>
+    <t>• Rule 92004 embeds Sysmon command-shell process creation with PowerShell parent
+• Rule 92217 records MpCmdRun.exe writing mpam-bce1d755.exe and UpdatePlatform.exe beneath C:\Windows\SystemTemp</t>
   </si>
 </sst>
 </file>
@@ -782,7 +781,7 @@
         <v>32</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="5" customFormat="1" ht="145.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
@@ -799,7 +798,7 @@
         <v>34</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="5" customFormat="1" ht="115.2" x14ac:dyDescent="0.3">
@@ -816,7 +815,7 @@
         <v>36</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="5" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
@@ -833,10 +832,10 @@
         <v>38</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" s="5" customFormat="1" ht="101.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" s="5" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A13" s="12" t="s">
         <v>20</v>
       </c>
@@ -844,13 +843,13 @@
         <v>25</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="5" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
@@ -861,13 +860,13 @@
         <v>26</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.3">

</xml_diff>